<commit_message>
Added heat map app
</commit_message>
<xml_diff>
--- a/Pathways Update/PathwaysAdd.xlsx
+++ b/Pathways Update/PathwaysAdd.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zaksprowls/Desktop/SPCAAutomation/Pathways Update/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{900CCAA8-12A3-9D4C-A1B2-EE054375CFF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E6A83A-C1ED-B445-8A1D-023A80254D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="0" windowWidth="19480" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -791,24 +791,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4CFF92"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -838,13 +826,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1399,60 +1386,60 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="2">
         <v>71.5</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="2">
         <v>71.5</v>
       </c>
     </row>
@@ -1486,60 +1473,60 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="2">
         <v>62.5</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="2">
         <v>66.5</v>
       </c>
     </row>
@@ -1689,60 +1676,60 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="H19" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I19" s="3">
+      <c r="I19" s="2">
         <v>30.5</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="H20" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="I20" s="3">
+      <c r="I20" s="2">
         <v>30.5</v>
       </c>
     </row>
@@ -1863,118 +1850,118 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="F25" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="G25" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="H25" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="I25" s="3">
+      <c r="I25" s="2">
         <v>31.6</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="F26" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G26" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="H26" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I26" s="3">
+      <c r="I26" s="2">
         <v>72.3</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F27" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G27" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="H27" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="I27" s="3">
+      <c r="I27" s="2">
         <v>30.5</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F28" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="G28" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="H28" s="3" t="s">
+      <c r="H28" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="I28" s="3">
+      <c r="I28" s="2">
         <v>42.5</v>
       </c>
     </row>
@@ -2008,257 +1995,257 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F30" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="G30" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="H30" s="3" t="s">
+      <c r="H30" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I30" s="3">
+      <c r="I30" s="2">
         <v>52.5</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F31" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G31" s="3" t="s">
+      <c r="G31" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="H31" s="3" t="s">
+      <c r="H31" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I31" s="3">
+      <c r="I31" s="2">
         <v>52.5</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="F32" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="G32" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="H32" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I32" s="3">
+      <c r="I32" s="2">
         <v>52.5</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="F33" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="G33" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="H33" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I33" s="3">
+      <c r="I33" s="2">
         <v>52.5</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="F34" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="G34" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="H34" s="3" t="s">
+      <c r="H34" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I34" s="3">
+      <c r="I34" s="2">
         <v>38.4</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3" t="s">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="F35" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G35" s="3" t="s">
+      <c r="G35" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="H35" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I35" s="3">
+      <c r="I35" s="2">
         <v>38.4</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3" t="s">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="F36" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G36" s="3" t="s">
+      <c r="G36" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="H36" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I36" s="3">
+      <c r="I36" s="2">
         <v>38.4</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3" t="s">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F37" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G37" s="3" t="s">
+      <c r="G37" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="H37" s="3" t="s">
+      <c r="H37" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I37" s="3">
+      <c r="I37" s="2">
         <v>38.4</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="F38" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G38" s="3" t="s">
+      <c r="G38" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="H38" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I38" s="3">
+      <c r="I38" s="2">
         <v>38.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated files for 7/8/25
</commit_message>
<xml_diff>
--- a/Pathways Update/PathwaysAdd.xlsx
+++ b/Pathways Update/PathwaysAdd.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,12 +478,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Marble</t>
+          <t>Trivento</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>57806699</t>
+          <t>58448688</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -493,42 +493,42 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Cat Adoption Room G</t>
+          <t>Cat Adoption Condo Rooms</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>04/28/2025</t>
+          <t>05/06/2025</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Domestic Shorthair</t>
+          <t>Domestic Longhair</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2y 3m 17d</t>
+          <t>2y 2m 1d</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Hold - Behavior Mod.</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>63</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FRANKLIN</t>
+          <t>CHATEAU ST. MICHELLE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>58365909</t>
+          <t>58459452</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -538,42 +538,42 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>If The Fur Fits</t>
+          <t>Cat Adoption Condo Rooms</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>04/29/2025</t>
+          <t>05/08/2025</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Domestic Shorthair</t>
+          <t>Domestic Longhair</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>8y 2m 6d</t>
+          <t>3y 2m 0d</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>In If the Fur Fits - Medical</t>
+          <t>Hold - Behavior Mod.</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>61.8</v>
+        <v>60.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PLUM</t>
+          <t>BEATRICE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>58377570</t>
+          <t>58442198</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -583,42 +583,42 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>If The Fur Fits</t>
+          <t>Foster Home</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>04/25/2025</t>
+          <t>05/06/2025</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Domestic Longhair</t>
+          <t>Domestic Shorthair</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>7y 2m 4d</t>
+          <t>2y 2m 1d</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>In If the Fur Fits - Medical</t>
+          <t>In Foster</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>65.7</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mochi</t>
+          <t>Sam</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>58353916</t>
+          <t>58444073</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -628,267 +628,263 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Offsite Adoptions</t>
+          <t>Foster Home</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>04/22/2025</t>
+          <t>05/06/2025</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Domestic Longhair</t>
+          <t>Domestic Shorthair</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2m 29d</t>
+          <t>3m 0d</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>In Foster</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>68.7</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CARAMEL</t>
+          <t>Masie</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>58640671</t>
+          <t>58450156</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Cat</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Adoptions Office (Jill's) #152</t>
+          <t>Foster Home</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>06/04/2025</t>
+          <t>05/07/2025</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Mixed Breed, Medium (up to 44 lbs fully grown)</t>
+          <t>Domestic Longhair</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5y 1m 15d</t>
+          <t>1y 8m 1d</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Hold - Behavior Mod.</t>
+          <t>In Foster</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>25.8</v>
+        <v>61.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SUDS</t>
+          <t>Quinta Nova</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>58598619</t>
+          <t>58454445</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Cat</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Dog Adoptions A</t>
+          <t>If The Fur Fits</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>05/29/2025</t>
+          <t>05/07/2025</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Chihuahua, Short Coat</t>
+          <t>Domestic Longhair</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5y 1m 1d</t>
+          <t>2y 2m 1d</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Available - Behind the Scenes</t>
+          <t>In If the Fur Fits - Behavior</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>31.8</v>
+        <v>61.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Charles</t>
+          <t>Momo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>58604196</t>
+          <t>58448506</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Cat</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Dog Adoptions A</t>
+          <t>If The Fur Fits</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>05/30/2025</t>
+          <t>05/06/2025</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Mixed Breed, Large (over 44 lbs fully grown)</t>
+          <t>Ragdoll</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5y 1m 0d</t>
+          <t>4m 12d</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Available - Behind the Scenes</t>
+          <t>In If the Fur Fits - Medical</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>31</v>
+        <v>62.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Benji</t>
+          <t>Elvis</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>58639325</t>
+          <t>58452209</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Cat</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Dog Adoptions A</t>
+          <t>If The Fur Fits</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>06/04/2025</t>
+          <t>05/07/2025</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Mixed Breed, Large (over 44 lbs fully grown)</t>
+          <t>Domestic Shorthair</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>10y 26d</t>
+          <t>1y 2m 1d</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Available - Behind the Scenes</t>
+          <t>In If the Fur Fits - Medical</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>25.8</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Pancake</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>58596028</t>
+          <t>58447679</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Cat</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Dog Adoptions B</t>
+          <t>If The Fur Fits</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>06/05/2025</t>
+          <t>05/06/2025</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Mixed Breed, Medium (up to 44 lbs fully grown)</t>
+          <t>Snowshoe</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3y 25d</t>
+          <t>3m 7d</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>In If the Fur Fits - Trial</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>24.9</v>
+        <v>62.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Snow Cone</t>
+          <t>Missy</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>58640624</t>
+          <t>58764565</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -898,42 +894,42 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Dog Adoptions C</t>
+          <t>Dog Adoptions B</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>06/04/2025</t>
+          <t>06/23/2025</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Mixed Breed, Medium (up to 44 lbs fully grown)</t>
+          <t>Mixed Breed, Large (over 44 lbs fully grown)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5y 1m 6d</t>
+          <t>3y 14d</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Hold - Meet and Greet</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>25.8</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Goldie</t>
+          <t>Karma</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>58622481</t>
+          <t>58764550</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -943,12 +939,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Dog Adoptions C</t>
+          <t>Dog Adoptions B</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>06/02/2025</t>
+          <t>06/23/2025</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -958,27 +954,27 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>7y 6m 19d</t>
+          <t>2y 15d</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Hold - Meet and Greet</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>27.8</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Beau</t>
+          <t>Onyx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>58677023</t>
+          <t>58622436</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -988,42 +984,42 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Dog Adoptions C</t>
+          <t>Dog Adoptions D</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>06/21/2025</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Mixed Breed, Large (over 44 lbs fully grown)</t>
+          <t>Shepherd</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2y 20d</t>
+          <t>6y 1m 6d</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Available - ITFF Behavior</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>19.9</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Maya</t>
+          <t>CINDER</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>58703260</t>
+          <t>58753979</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1038,7 +1034,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>06/13/2025</t>
+          <t>06/20/2025</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1048,27 +1044,27 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>11y 17d</t>
+          <t>10y 4m 10d</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Hold - Doc</t>
+          <t>Hold - Rescue</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>16.9</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Iris</t>
+          <t>Diamond</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>58545411</t>
+          <t>57957792</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1078,12 +1074,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Foster Home</t>
+          <t>Dog Holding F</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>05/27/2025</t>
+          <t>03/04/2025</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1093,27 +1089,27 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10m 2d</t>
+          <t>1y 1m 26d</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>In Foster</t>
+          <t>Hold - Behavior</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>33.9</v>
+        <v>125.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pickley</t>
+          <t>EASTON</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>58605268</t>
+          <t>58718199</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1123,42 +1119,42 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Foster Home</t>
+          <t>If The Fur Fits</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>05/31/2025</t>
+          <t>06/18/2025</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Poodle, Standard</t>
+          <t>Mixed Breed, Medium (up to 44 lbs fully grown)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4y 1m 0d</t>
+          <t>8y 2m 0d</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>In SAFE Foster</t>
+          <t>In If the Fur Fits - Medical</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>29.9</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>THOR</t>
+          <t>Magnus</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>32144299</t>
+          <t>58690617</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1173,37 +1169,37 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>06/09/2025</t>
+          <t>06/19/2025</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Collie, Smooth</t>
+          <t>Mixed Breed, Large (over 44 lbs fully grown)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>9y 5m 17d</t>
+          <t>4y 27d</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>In If the Fur Fits - Medical</t>
+          <t>In If the Fur Fits - Trial</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>20.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bubba</t>
+          <t>JEWELIE</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>57976477</t>
+          <t>58753970</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1218,172 +1214,168 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>06/06/2025</t>
+          <t>06/20/2025</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Mixed Breed, Large (over 44 lbs fully grown)</t>
+          <t>Mixed Breed, Small (under 24 lbs fully grown)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>11m 23d</t>
+          <t>10y 17d</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>In If the Fur Fits - Medical</t>
+          <t>In If the Fur Fits - Trial</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>24</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bella</t>
+          <t>FIREFLY</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>58597214</t>
+          <t>58695418</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Rabbit</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>If The Fur Fits</t>
+          <t>Cat Adoption Condo Rooms</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>06/03/2025</t>
+          <t>06/20/2025</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Mixed Breed, Medium (up to 44 lbs fully grown)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>5y 1m 1d</t>
-        </is>
-      </c>
+          <t>Mix</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>In If the Fur Fits - Medical</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>26.9</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RAYNE</t>
+          <t>Luna</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>57710656</t>
+          <t>58744079</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Donkey</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>If The Fur Fits</t>
+          <t>Farm</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>06/13/2025</t>
+          <t>06/17/2025</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Mixed Breed, Large (over 44 lbs fully grown)</t>
+          <t>Miniature Donkey</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>4y 5m 6d</t>
+          <t>15y 19d</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>In If the Fur Fits - Trial</t>
+          <t>Hold - Doc</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>16.8</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HEATH</t>
+          <t>Moose</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>58654173</t>
+          <t>58728965</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Farm Type Fowl</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>If The Fur Fits</t>
+          <t>Farm</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>06/06/2025</t>
+          <t>06/17/2025</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Whippet</t>
+          <t>Chicken</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>7m 26d</t>
+          <t>8m 23d</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>In If the Fur Fits - Trial</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>23.9</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MARINA</t>
+          <t>FUZZY SLIPPER</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>58706705</t>
+          <t>58757630</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1393,79 +1385,87 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Adoptions Lobby</t>
+          <t>Foster Home</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>06/13/2025</t>
+          <t>06/21/2025</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>Mini-Lop</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2m 29d</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>In Foster</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>16.8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>FLIP FLOP</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>58757640</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Rabbit</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Foster Home</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>06/21/2025</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>Rex</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>16.7</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>58654136</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Domestic (Cage) Bird</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Farm</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>06/06/2025</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Quail, Japanese</t>
-        </is>
-      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>3m 3d</t>
+          <t>2m 29d</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>In Foster</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>23.9</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Bunny 2</t>
+          <t>Leonardo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>58212975</t>
+          <t>58764920</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1480,17 +1480,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>03/30/2025</t>
+          <t>06/23/2025</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Florida White</t>
+          <t>Satin</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3m 1d</t>
+          <t>1y 15d</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1499,498 +1499,7 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Bunny 1</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>58212978</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Florida White</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Glacier</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>58212979</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Florida White</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Apple</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>58212981</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Florida White</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Cloudy</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>58212982</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Florida White</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Bunny 5</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>58212985</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Florida White</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Bunny 7</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>58212987</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Florida White</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Ham</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>58213029</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Rex</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Rabbit 1</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>58213031</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Rex</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Rabbit 4</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>58213033</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Rex</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Jam</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>58213035</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Rex</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>91.90000000000001</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>58213036</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Rabbit</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Foster Home</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>03/30/2025</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Rex</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>3m 1d</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>In Foster</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>91.90000000000001</v>
+        <v>14.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>